<commit_message>
fix(workbook): categorías de texto con strRef en gráficos 3, 4 y 5
openpyxl.set_categories escribe numRef incluso para etiquetas de texto.
Los gráficos de comparativa, productos y costes usan ahora AxDataSource/StrRef;
los gráficos mensuales mantienen numRef para sus fechas.
</commit_message>
<xml_diff>
--- a/docs/assets/Cafeteria-Aurora-Modelo-Financiero.xlsx
+++ b/docs/assets/Cafeteria-Aurora-Modelo-Financiero.xlsx
@@ -909,9 +909,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumen'!$A$151:$A$153</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -936,9 +936,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumen'!$A$151:$A$153</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -963,9 +963,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumen'!$A$151:$A$153</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1066,9 +1066,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumen'!$B$158:$B$165</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1162,9 +1162,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'Resumen'!$B$169:$B$173</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>

</xml_diff>